<commit_message>
Updates for Spring 2026
</commit_message>
<xml_diff>
--- a/people.xlsx
+++ b/people.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jessicaalexander/github/rlp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{956D8AE0-7D27-BB43-B28E-A869B6C0B17D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92248EE3-C2B6-AF4E-B7A2-CC87E8197384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7620" yWindow="680" windowWidth="20820" windowHeight="15900" xr2:uid="{59A264FB-7A95-E842-AEEA-C35557593B53}"/>
+    <workbookView xWindow="7620" yWindow="680" windowWidth="20820" windowHeight="15820" xr2:uid="{59A264FB-7A95-E842-AEEA-C35557593B53}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -88,9 +88,6 @@
     <t>Deshpande</t>
   </si>
   <si>
-    <t>W5</t>
-  </si>
-  <si>
     <t>Qing</t>
   </si>
   <si>
@@ -130,15 +127,6 @@
     <t>W10</t>
   </si>
   <si>
-    <t>Taylor</t>
-  </si>
-  <si>
-    <t>Joyce</t>
-  </si>
-  <si>
-    <t>W11</t>
-  </si>
-  <si>
     <t>Barrett</t>
   </si>
   <si>
@@ -589,10 +577,22 @@
     <t>WCP 4.134</t>
   </si>
   <si>
-    <t>4.110/W8</t>
-  </si>
-  <si>
     <t>Thiago</t>
+  </si>
+  <si>
+    <t>4.110/W11</t>
+  </si>
+  <si>
+    <t>4.434</t>
+  </si>
+  <si>
+    <t>4.110/W5</t>
+  </si>
+  <si>
+    <t>Sarah</t>
+  </si>
+  <si>
+    <t>Ransom Laud</t>
   </si>
 </sst>
 </file>
@@ -972,30 +972,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D2" s="4" t="str">
-        <f t="shared" ref="D2:D36" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
+        <f t="shared" ref="D2:D35" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
         <v>Akshay Aitha   4.706</v>
       </c>
     </row>
@@ -1007,22 +1007,22 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>4</v>
+        <v>183</v>
       </c>
       <c r="D3" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Jess Alexander   4.110</v>
+        <v>Jess Alexander   4.110/W5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D4" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1031,13 +1031,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D5" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1046,13 +1046,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D6" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1061,13 +1061,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D7" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1076,13 +1076,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B8" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D8" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1106,13 +1106,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B10" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D10" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1121,13 +1121,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B11" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D11" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1136,13 +1136,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D12" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1151,13 +1151,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B13" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D13" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1166,13 +1166,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B14" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D14" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1181,13 +1181,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B15" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D15" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1196,13 +1196,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B16" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D16" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1211,13 +1211,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B17" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D17" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1232,22 +1232,22 @@
         <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>17</v>
+        <v>182</v>
       </c>
       <c r="D18" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Sampada Deshpande   W5</v>
+        <v>Sampada Deshpande   4.434</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B19" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D19" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1256,13 +1256,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D20" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1271,13 +1271,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D21" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1286,13 +1286,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D22" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1301,13 +1301,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D23" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1316,13 +1316,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
         <v>28</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="D24" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1331,13 +1331,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D25" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1346,13 +1346,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B26" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D26" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1361,358 +1361,358 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>171</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>172</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="D27" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Taylor Joyce   W11</v>
+        <v>Anushri Kartik-Narajan   4.110</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>175</v>
+        <v>103</v>
       </c>
       <c r="B28" t="s">
-        <v>176</v>
+        <v>104</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>4</v>
+        <v>105</v>
       </c>
       <c r="D28" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Anushri Kartik-Narajan   4.110</v>
+        <v>Danny Law   4.432</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="D29" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Danny Law   4.432</v>
+        <v>Rebecca Le Borgne   4.624</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="B30" t="s">
-        <v>99</v>
+        <v>23</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>98</v>
+        <v>61</v>
       </c>
       <c r="D30" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Rebecca Le Borgne   4.624</v>
+        <v>Sooji Lee   E6</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>64</v>
+        <v>135</v>
       </c>
       <c r="B31" t="s">
-        <v>24</v>
+        <v>136</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>65</v>
+        <v>137</v>
       </c>
       <c r="D31" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Sooji Lee   E6</v>
+        <v>Jessy Li   4.728</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
+        <v>138</v>
+      </c>
+      <c r="B32" t="s">
         <v>139</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>141</v>
-      </c>
       <c r="D32" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Jessy Li   4.728</v>
+        <v>Fernando Llanos   4.730</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>142</v>
+        <v>100</v>
       </c>
       <c r="B33" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>144</v>
+        <v>102</v>
       </c>
       <c r="D33" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Fernando Llanos   4.730</v>
+        <v>Kyle Mahowald   4.430</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>104</v>
+        <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>105</v>
+        <v>40</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>106</v>
+        <v>41</v>
       </c>
       <c r="D34" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Kyle Mahowald   4.430</v>
+        <v>Rebecca Marcus   4.304C</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>43</v>
+        <v>141</v>
       </c>
       <c r="B35" t="s">
-        <v>44</v>
+        <v>142</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>45</v>
+        <v>143</v>
       </c>
       <c r="D35" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Rebecca Marcus   4.304C</v>
+        <v>Richard Meier   4.732</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>145</v>
+        <v>82</v>
       </c>
       <c r="B36" t="s">
-        <v>146</v>
+        <v>83</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>147</v>
+        <v>84</v>
       </c>
       <c r="D36" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Richard Meier   4.732</v>
+        <f t="shared" ref="D36:D65" si="1">CONCATENATE(A36, " ", B36, "   ", C36)</f>
+        <v>Don Miller   4.618</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>160</v>
       </c>
       <c r="B37" t="s">
-        <v>87</v>
+        <v>161</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="D37" s="4" t="str">
-        <f t="shared" ref="D37:D65" si="1">CONCATENATE(A37, " ", B37, "   ", C37)</f>
-        <v>Don Miller   4.618</v>
+        <f t="shared" si="1"/>
+        <v>Kanishka Misra   4.428</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B38" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>103</v>
+        <v>5</v>
       </c>
       <c r="D38" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Kanishka Misra   4.428</v>
+        <v>Kaiji Mo   W1</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>169</v>
+        <v>132</v>
       </c>
       <c r="B39" t="s">
-        <v>170</v>
+        <v>133</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>5</v>
+        <v>134</v>
       </c>
       <c r="D39" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Kaiji Mo   W1</v>
+        <v>Scott Myers   4.726</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>136</v>
+        <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>137</v>
+        <v>37</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>138</v>
+        <v>38</v>
       </c>
       <c r="D40" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Scott Myers   4.726</v>
+        <v>Lillian Nguyen   FD</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>42</v>
+        <v>181</v>
       </c>
       <c r="D41" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lillian Nguyen   FD</v>
+        <v>Baorian Nuchged   4.110/W11</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="B42" t="s">
-        <v>1</v>
+        <v>158</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>184</v>
+        <v>144</v>
       </c>
       <c r="D42" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Baorian Nuchged   4.110/W8</v>
+        <v>Karol Obert   4.734</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>161</v>
+        <v>109</v>
       </c>
       <c r="B43" t="s">
-        <v>162</v>
+        <v>110</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>148</v>
+        <v>111</v>
       </c>
       <c r="D43" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Karol Obert   4.734</v>
+        <v>Corrine Occhino   4.704</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>113</v>
+        <v>23</v>
       </c>
       <c r="B44" t="s">
-        <v>114</v>
+        <v>24</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>115</v>
+        <v>25</v>
       </c>
       <c r="D44" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Corrine Occhino   4.704</v>
+        <v>Lee Orfila   W8</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D45" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lee Orfila   W8</v>
+        <v>Youn-Gyu Park   W7</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" t="s">
         <v>21</v>
       </c>
-      <c r="B46" t="s">
-        <v>22</v>
-      </c>
       <c r="C46" s="1" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="D46" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Youn-Gyu Park   W7</v>
+        <v>SeYeon Park   (NA)</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="B47" t="s">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>76</v>
+        <v>162</v>
       </c>
       <c r="D47" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>SeYeon Park   E10</v>
+        <v>Justin Power   4.740</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B48" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>166</v>
+        <v>122</v>
       </c>
       <c r="D48" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Justin Power   4.740</v>
+        <v>David Quinto-Pozos   4.714</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>119</v>
+        <v>184</v>
       </c>
       <c r="B49" t="s">
-        <v>125</v>
+        <v>185</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="D49" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>David Quinto-Pozos   4.714</v>
+        <v>Sarah Ransom Laud   (NA)</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B50" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D50" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1721,13 +1721,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B51" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D51" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1736,13 +1736,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B52" t="s">
+        <v>77</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="D52" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1751,13 +1751,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B53" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D53" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1766,13 +1766,13 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B54" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D54" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1796,13 +1796,13 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B56" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D56" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1817,22 +1817,22 @@
         <v>10</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="D57" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Madeline Smith   (NA)</v>
+        <v>Madeline Smith   E10</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B58" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D58" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1841,13 +1841,13 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B59" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D59" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1856,13 +1856,13 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B60" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D60" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1871,13 +1871,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B61" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D61" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1886,13 +1886,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B62" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D62" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1901,13 +1901,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
+        <v>17</v>
+      </c>
+      <c r="B63" t="s">
         <v>18</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="D63" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1916,13 +1916,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B64" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D64" s="4" t="str">
         <f t="shared" si="1"/>
@@ -1931,10 +1931,10 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B65" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Additional shifts for spring 2026
</commit_message>
<xml_diff>
--- a/people.xlsx
+++ b/people.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jessicaalexander/github/rlp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92248EE3-C2B6-AF4E-B7A2-CC87E8197384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{398306E1-85E5-4840-9D75-A15770556D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7620" yWindow="680" windowWidth="20820" windowHeight="15820" xr2:uid="{59A264FB-7A95-E842-AEEA-C35557593B53}"/>
+    <workbookView xWindow="7620" yWindow="680" windowWidth="20820" windowHeight="15740" xr2:uid="{59A264FB-7A95-E842-AEEA-C35557593B53}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="189">
   <si>
     <t>Baorian</t>
   </si>
@@ -593,6 +593,15 @@
   </si>
   <si>
     <t>Ransom Laud</t>
+  </si>
+  <si>
+    <t>W5</t>
+  </si>
+  <si>
+    <t>Caitlin</t>
+  </si>
+  <si>
+    <t>Coons</t>
   </si>
 </sst>
 </file>
@@ -963,7 +972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17483530-688E-B14A-9F3B-5498A1C19FFD}">
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="10.83203125" style="1"/>
@@ -995,7 +1004,7 @@
         <v>114</v>
       </c>
       <c r="D2" s="4" t="str">
-        <f t="shared" ref="D2:D35" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
+        <f t="shared" ref="D2:D36" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
         <v>Akshay Aitha   4.706</v>
       </c>
     </row>
@@ -1181,772 +1190,787 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>118</v>
+        <v>187</v>
       </c>
       <c r="B15" t="s">
-        <v>119</v>
+        <v>188</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>120</v>
+        <v>72</v>
       </c>
       <c r="D15" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Megan Crowhurst   4.712</v>
+        <v>Caitlin Coons   E10</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>156</v>
+        <v>118</v>
       </c>
       <c r="B16" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>179</v>
+        <v>120</v>
       </c>
       <c r="D16" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Meg Davidson   WCP 4.134</v>
+        <v>Megan Crowhurst   4.712</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>96</v>
+        <v>156</v>
       </c>
       <c r="B17" t="s">
-        <v>97</v>
+        <v>155</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>98</v>
+        <v>179</v>
       </c>
       <c r="D17" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Ashwini Deo   4.426</v>
+        <v>Meg Davidson   WCP 4.134</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>96</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>97</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>182</v>
+        <v>98</v>
       </c>
       <c r="D18" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Sampada Deshpande   4.434</v>
+        <v>Ashwini Deo   4.426</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>146</v>
+        <v>16</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>147</v>
+        <v>182</v>
       </c>
       <c r="D19" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Pattie Epps   4.736</v>
+        <v>Sampada Deshpande   4.434</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>145</v>
       </c>
       <c r="B20" t="s">
-        <v>63</v>
+        <v>146</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>64</v>
+        <v>147</v>
       </c>
       <c r="D20" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Teagan Esther   E7</v>
+        <v>Pattie Epps   4.736</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="D21" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>James Fazio   4.622</v>
+        <v>Teagan Esther   E7</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="B22" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="D22" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Gabriel Gallinate   E8</v>
+        <v>James Fazio   4.622</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>32</v>
+        <v>67</v>
       </c>
       <c r="D23" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Barrett Hamp   W12</v>
+        <v>Gabriel Gallinate   E8</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D24" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Leticia Hanada   W10</v>
+        <v>Barrett Hamp   W12</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="D25" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Ethan Hartzell   E3</v>
+        <v>Leticia Hanada   W10</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>173</v>
+        <v>51</v>
       </c>
       <c r="B26" t="s">
-        <v>174</v>
+        <v>52</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="D26" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Juan Pablo Jáuregui Magrina   (NA)</v>
+        <v>Ethan Hartzell   E3</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B27" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="D27" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Anushri Kartik-Narajan   4.110</v>
+        <v>Juan Pablo Jáuregui Magrina   (NA)</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>103</v>
+        <v>171</v>
       </c>
       <c r="B28" t="s">
-        <v>104</v>
+        <v>172</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>105</v>
+        <v>4</v>
       </c>
       <c r="D28" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Danny Law   4.432</v>
+        <v>Anushri Kartik-Narajan   4.110</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>39</v>
+        <v>103</v>
       </c>
       <c r="B29" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="D29" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Rebecca Le Borgne   4.624</v>
+        <v>Danny Law   4.432</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>23</v>
+        <v>95</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="D30" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Sooji Lee   E6</v>
+        <v>Rebecca Le Borgne   4.624</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="B31" t="s">
-        <v>136</v>
+        <v>23</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>137</v>
+        <v>61</v>
       </c>
       <c r="D31" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Jessy Li   4.728</v>
+        <v>Sooji Lee   E6</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B32" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D32" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Fernando Llanos   4.730</v>
+        <v>Jessy Li   4.728</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="B33" t="s">
-        <v>101</v>
+        <v>139</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>102</v>
+        <v>140</v>
       </c>
       <c r="D33" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Kyle Mahowald   4.430</v>
+        <v>Fernando Llanos   4.730</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>101</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="D34" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Rebecca Marcus   4.304C</v>
+        <v>Kyle Mahowald   4.430</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>141</v>
+        <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>142</v>
+        <v>40</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>143</v>
+        <v>41</v>
       </c>
       <c r="D35" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Richard Meier   4.732</v>
+        <v>Rebecca Marcus   4.304C</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>82</v>
+        <v>141</v>
       </c>
       <c r="B36" t="s">
-        <v>83</v>
+        <v>142</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>84</v>
+        <v>143</v>
       </c>
       <c r="D36" s="4" t="str">
-        <f t="shared" ref="D36:D65" si="1">CONCATENATE(A36, " ", B36, "   ", C36)</f>
-        <v>Don Miller   4.618</v>
+        <f t="shared" si="0"/>
+        <v>Richard Meier   4.732</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>160</v>
+        <v>82</v>
       </c>
       <c r="B37" t="s">
-        <v>161</v>
+        <v>83</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="D37" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Kanishka Misra   4.428</v>
+        <f t="shared" ref="D37:D66" si="1">CONCATENATE(A37, " ", B37, "   ", C37)</f>
+        <v>Don Miller   4.618</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B38" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="D38" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Kaiji Mo   W1</v>
+        <v>Kanishka Misra   4.428</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>132</v>
+        <v>165</v>
       </c>
       <c r="B39" t="s">
-        <v>133</v>
+        <v>166</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>134</v>
+        <v>5</v>
       </c>
       <c r="D39" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Scott Myers   4.726</v>
+        <v>Kaiji Mo   W1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>36</v>
+        <v>132</v>
       </c>
       <c r="B40" t="s">
-        <v>37</v>
+        <v>133</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>38</v>
+        <v>134</v>
       </c>
       <c r="D40" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lillian Nguyen   FD</v>
+        <v>Scott Myers   4.726</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="B41" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>181</v>
+        <v>38</v>
       </c>
       <c r="D41" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Baorian Nuchged   4.110/W11</v>
+        <v>Lillian Nguyen   FD</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="B42" t="s">
-        <v>158</v>
+        <v>1</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>144</v>
+        <v>181</v>
       </c>
       <c r="D42" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Karol Obert   4.734</v>
+        <v>Baorian Nuchged   4.110/W11</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>109</v>
+        <v>157</v>
       </c>
       <c r="B43" t="s">
-        <v>110</v>
+        <v>158</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>111</v>
+        <v>144</v>
       </c>
       <c r="D43" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Corrine Occhino   4.704</v>
+        <v>Karol Obert   4.734</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>23</v>
+        <v>109</v>
       </c>
       <c r="B44" t="s">
-        <v>24</v>
+        <v>110</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>25</v>
+        <v>111</v>
       </c>
       <c r="D44" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lee Orfila   W8</v>
+        <v>Corrine Occhino   4.704</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B45" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D45" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Youn-Gyu Park   W7</v>
+        <v>Lee Orfila   W8</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="B46" t="s">
         <v>21</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="D46" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>SeYeon Park   (NA)</v>
+        <v>Youn-Gyu Park   W7</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>112</v>
+        <v>71</v>
       </c>
       <c r="B47" t="s">
-        <v>113</v>
+        <v>21</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>162</v>
+        <v>80</v>
       </c>
       <c r="D47" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Justin Power   4.740</v>
+        <v>SeYeon Park   (NA)</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B48" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>122</v>
+        <v>162</v>
       </c>
       <c r="D48" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>David Quinto-Pozos   4.714</v>
+        <v>Justin Power   4.740</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>184</v>
+        <v>115</v>
       </c>
       <c r="B49" t="s">
-        <v>185</v>
+        <v>121</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>80</v>
+        <v>122</v>
       </c>
       <c r="D49" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Sarah Ransom Laud   (NA)</v>
+        <v>David Quinto-Pozos   4.714</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>42</v>
+        <v>184</v>
       </c>
       <c r="B50" t="s">
-        <v>43</v>
+        <v>185</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D50" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Ben Rapstine   4.304D</v>
+        <v>Sarah Ransom Laud   (NA)</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>175</v>
+        <v>42</v>
       </c>
       <c r="B51" t="s">
-        <v>176</v>
+        <v>43</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D51" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Oscar Rojas   E8</v>
+        <v>Ben Rapstine   4.304D</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>76</v>
+        <v>175</v>
       </c>
       <c r="B52" t="s">
-        <v>77</v>
+        <v>176</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="D52" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Catalina Santamaria Soto   E12</v>
+        <v>Oscar Rojas   E8</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
       <c r="B53" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="D53" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Jefferson Saransig   W13</v>
+        <v>Catalina Santamaria Soto   E12</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>167</v>
+        <v>33</v>
       </c>
       <c r="B54" t="s">
-        <v>168</v>
+        <v>34</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="D54" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Ari Schifman   E2</v>
+        <v>Jefferson Saransig   W13</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>12</v>
+        <v>167</v>
       </c>
       <c r="B55" t="s">
-        <v>13</v>
+        <v>168</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="D55" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Will Sheffield   W4</v>
+        <v>Ari Schifman   E2</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>129</v>
+        <v>12</v>
       </c>
       <c r="B56" t="s">
-        <v>130</v>
+        <v>13</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>131</v>
+        <v>14</v>
       </c>
       <c r="D56" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Rajka Smiljanić   4.724</v>
+        <v>Will Sheffield   W4</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>9</v>
+        <v>129</v>
       </c>
       <c r="B57" t="s">
-        <v>10</v>
+        <v>130</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>72</v>
+        <v>131</v>
       </c>
       <c r="D57" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Madeline Smith   E10</v>
+        <v>Rajka Smiljanić   4.724</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>106</v>
+        <v>9</v>
       </c>
       <c r="B58" t="s">
-        <v>107</v>
+        <v>10</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>108</v>
+        <v>186</v>
       </c>
       <c r="D58" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Steve Wechsler   4.702</v>
+        <v>Madeline Smith   W5</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
       <c r="B59" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="D59" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Debbie White   4.620</v>
+        <v>Steve Wechsler   4.702</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="B60" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D60" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Elijah Wilder   E11</v>
+        <v>Debbie White   4.620</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>148</v>
+        <v>73</v>
       </c>
       <c r="B61" t="s">
-        <v>149</v>
+        <v>74</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="D61" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Tony Woodbury   4.738</v>
+        <v>Elijah Wilder   E11</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>91</v>
+        <v>148</v>
       </c>
       <c r="B62" t="s">
-        <v>92</v>
+        <v>149</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>93</v>
+        <v>150</v>
       </c>
       <c r="D62" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Michael Wynne   4.626</v>
+        <v>Tony Woodbury   4.738</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>17</v>
+        <v>91</v>
       </c>
       <c r="B63" t="s">
-        <v>18</v>
+        <v>92</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>19</v>
+        <v>93</v>
       </c>
       <c r="D63" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Qing Yao   W6</v>
+        <v>Michael Wynne   4.626</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>78</v>
+        <v>17</v>
       </c>
       <c r="B64" t="s">
-        <v>79</v>
+        <v>18</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>80</v>
+        <v>19</v>
       </c>
       <c r="D64" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Hongli Zhan   (NA)</v>
+        <v>Qing Yao   W6</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
+        <v>78</v>
+      </c>
+      <c r="B65" t="s">
+        <v>79</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D65" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Hongli Zhan   (NA)</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
         <v>45</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B66" t="s">
         <v>46</v>
       </c>
-      <c r="C65" s="1" t="s">
+      <c r="C66" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D65" s="4" t="str">
+      <c r="D66" s="4" t="str">
         <f t="shared" si="1"/>
         <v>Asher Zheng   W3</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D65">
-    <sortCondition ref="B3:B65"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D66">
+    <sortCondition ref="B3:B66"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update labs and offices for Fall 2026
</commit_message>
<xml_diff>
--- a/people.xlsx
+++ b/people.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jessicaalexander/github/rlp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE9491DC-EA9D-6E4A-A8D1-32EC422FBB24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF6C52CD-C44F-2345-99A3-618B6A795643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7620" yWindow="680" windowWidth="20820" windowHeight="15740" xr2:uid="{59A264FB-7A95-E842-AEEA-C35557593B53}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="183">
   <si>
     <t>Baorian</t>
   </si>
@@ -325,15 +325,6 @@
     <t>Le Borgne</t>
   </si>
   <si>
-    <t>Ashwini</t>
-  </si>
-  <si>
-    <t>Deo</t>
-  </si>
-  <si>
-    <t>4.426</t>
-  </si>
-  <si>
     <t>4.428</t>
   </si>
   <si>
@@ -373,12 +364,6 @@
     <t>4.704</t>
   </si>
   <si>
-    <t>Justin</t>
-  </si>
-  <si>
-    <t>Power</t>
-  </si>
-  <si>
     <t>4.706</t>
   </si>
   <si>
@@ -521,9 +506,6 @@
   </si>
   <si>
     <t>Misra</t>
-  </si>
-  <si>
-    <t>4.740</t>
   </si>
   <si>
     <t>Akshay</t>
@@ -972,7 +954,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17483530-688E-B14A-9F3B-5498A1C19FFD}">
-  <dimension ref="A1:D66"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="10.83203125" style="1"/>
@@ -981,30 +963,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B2" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D2" s="4" t="str">
-        <f t="shared" ref="D2:D36" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
+        <f t="shared" ref="D2:D35" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
         <v>Akshay Aitha   4.706</v>
       </c>
     </row>
@@ -1016,7 +998,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D3" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1025,13 +1007,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B4" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D4" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1070,13 +1052,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B7" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D7" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1085,13 +1067,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="D8" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1115,10 +1097,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B10" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>38</v>
@@ -1130,10 +1112,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B11" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>26</v>
@@ -1160,10 +1142,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B13" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>80</v>
@@ -1190,10 +1172,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="B15" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>72</v>
@@ -1205,13 +1187,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B16" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="D16" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1220,13 +1202,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B17" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D17" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1235,742 +1217,712 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>96</v>
+        <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>97</v>
+        <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>98</v>
+        <v>175</v>
       </c>
       <c r="D18" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Ashwini Deo   4.426</v>
+        <v>Sampada Deshpande   4.434</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>140</v>
       </c>
       <c r="B19" t="s">
-        <v>16</v>
+        <v>141</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>181</v>
+        <v>142</v>
       </c>
       <c r="D19" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Sampada Deshpande   4.434</v>
+        <v>Pattie Epps   4.736</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>145</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s">
-        <v>146</v>
+        <v>63</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>147</v>
+        <v>64</v>
       </c>
       <c r="D20" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Pattie Epps   4.736</v>
+        <v>Teagan Esther   E7</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="D21" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Teagan Esther   E7</v>
+        <v>James Fazio   4.622</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="D22" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>James Fazio   4.622</v>
+        <v>Gabriel Gallinate   E8</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="D23" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Gabriel Gallinate   E8</v>
+        <v>Barrett Hamp   W12</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D24" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Barrett Hamp   W12</v>
+        <v>Leticia Hanada   W10</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="D25" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Leticia Hanada   W10</v>
+        <v>Ethan Hartzell   E3</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>166</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>167</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="D26" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Ethan Hartzell   E3</v>
+        <v>Juan Pablo Jáuregui Magrina   (NA)</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B27" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="D27" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Juan Pablo Jáuregui Magrina   (NA)</v>
+        <v>Anushri Kartik-Narajan   4.110</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>170</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
-        <v>171</v>
+        <v>101</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="D28" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Anushri Kartik-Narajan   4.110</v>
+        <v>Danny Law   4.432</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>103</v>
+        <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="D29" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Danny Law   4.432</v>
+        <v>Rebecca Le Borgne   4.624</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="B30" t="s">
-        <v>95</v>
+        <v>23</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="D30" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Rebecca Le Borgne   4.624</v>
+        <v>Sooji Lee   E6</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="B31" t="s">
-        <v>23</v>
+        <v>131</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>61</v>
+        <v>132</v>
       </c>
       <c r="D31" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Sooji Lee   E6</v>
+        <v>Jessy Li   4.728</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" t="s">
+        <v>134</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B32" t="s">
-        <v>136</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>137</v>
-      </c>
       <c r="D32" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Jessy Li   4.728</v>
+        <v>Fernando Llanos   4.730</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>138</v>
+        <v>97</v>
       </c>
       <c r="B33" t="s">
-        <v>139</v>
+        <v>98</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>140</v>
+        <v>99</v>
       </c>
       <c r="D33" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Fernando Llanos   4.730</v>
+        <v>Kyle Mahowald   4.430</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>100</v>
+        <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>101</v>
+        <v>40</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>102</v>
+        <v>41</v>
       </c>
       <c r="D34" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Kyle Mahowald   4.430</v>
+        <v>Rebecca Marcus   4.304C</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>136</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>137</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>41</v>
+        <v>138</v>
       </c>
       <c r="D35" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Rebecca Marcus   4.304C</v>
+        <v>Richard Meier   4.732</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>141</v>
+        <v>82</v>
       </c>
       <c r="B36" t="s">
-        <v>142</v>
+        <v>83</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>143</v>
+        <v>84</v>
       </c>
       <c r="D36" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Richard Meier   4.732</v>
+        <f t="shared" ref="D36:D64" si="1">CONCATENATE(A36, " ", B36, "   ", C36)</f>
+        <v>Don Miller   4.618</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>82</v>
+        <v>155</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>156</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="D37" s="4" t="str">
-        <f t="shared" ref="D37:D66" si="1">CONCATENATE(A37, " ", B37, "   ", C37)</f>
-        <v>Don Miller   4.618</v>
+        <f t="shared" si="1"/>
+        <v>Kanishka Misra   4.428</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>160</v>
+        <v>182</v>
       </c>
       <c r="B38" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>99</v>
+        <v>5</v>
       </c>
       <c r="D38" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Kanishka Misra   4.428</v>
+        <v>Kaijie Mo   W1</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>188</v>
+        <v>127</v>
       </c>
       <c r="B39" t="s">
-        <v>165</v>
+        <v>128</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>5</v>
+        <v>129</v>
       </c>
       <c r="D39" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Kaijie Mo   W1</v>
+        <v>Scott Myers   4.726</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>132</v>
+        <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>133</v>
+        <v>37</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>134</v>
+        <v>38</v>
       </c>
       <c r="D40" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Scott Myers   4.726</v>
+        <v>Lillian Nguyen   FD</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>38</v>
+        <v>174</v>
       </c>
       <c r="D41" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lillian Nguyen   FD</v>
+        <v>Baorian Nuchged   4.110/W11</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="B42" t="s">
-        <v>1</v>
+        <v>153</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>180</v>
+        <v>139</v>
       </c>
       <c r="D42" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Baorian Nuchged   4.110/W11</v>
+        <v>Karol Obert   4.734</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>157</v>
+        <v>106</v>
       </c>
       <c r="B43" t="s">
-        <v>158</v>
+        <v>107</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>144</v>
+        <v>108</v>
       </c>
       <c r="D43" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Karol Obert   4.734</v>
+        <v>Corrine Occhino   4.704</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>109</v>
+        <v>23</v>
       </c>
       <c r="B44" t="s">
-        <v>110</v>
+        <v>24</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>111</v>
+        <v>25</v>
       </c>
       <c r="D44" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Corrine Occhino   4.704</v>
+        <v>Lee Orfila   W8</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D45" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lee Orfila   W8</v>
+        <v>Youn-Gyu Park   W7</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="B46" t="s">
         <v>21</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="D46" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Youn-Gyu Park   W7</v>
+        <v>SeYeon Park   (NA)</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>71</v>
+        <v>110</v>
       </c>
       <c r="B47" t="s">
-        <v>21</v>
+        <v>116</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="D47" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>SeYeon Park   (NA)</v>
+        <v>David Quinto-Pozos   4.714</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>112</v>
+        <v>177</v>
       </c>
       <c r="B48" t="s">
-        <v>113</v>
+        <v>178</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>162</v>
+        <v>80</v>
       </c>
       <c r="D48" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Justin Power   4.740</v>
+        <v>Sarah Ransom Laud   (NA)</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>115</v>
+        <v>42</v>
       </c>
       <c r="B49" t="s">
-        <v>121</v>
+        <v>43</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>122</v>
+        <v>44</v>
       </c>
       <c r="D49" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>David Quinto-Pozos   4.714</v>
+        <v>Ben Rapstine   4.304D</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="B50" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="D50" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Sarah Ransom Laud   (NA)</v>
+        <v>Oscar Rojas   E8</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="B51" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="D51" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Ben Rapstine   4.304D</v>
+        <v>Catalina Santamaria Soto   E12</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>174</v>
+        <v>33</v>
       </c>
       <c r="B52" t="s">
-        <v>175</v>
+        <v>34</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="D52" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Oscar Rojas   E8</v>
+        <v>Jefferson Saransig   W13</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>76</v>
+        <v>160</v>
       </c>
       <c r="B53" t="s">
-        <v>77</v>
+        <v>161</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>81</v>
+        <v>50</v>
       </c>
       <c r="D53" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Catalina Santamaria Soto   E12</v>
+        <v>Ari Schifman   E2</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="B54" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="D54" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Jefferson Saransig   W13</v>
+        <v>Will Sheffield   W4</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>166</v>
+        <v>124</v>
       </c>
       <c r="B55" t="s">
-        <v>167</v>
+        <v>125</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>50</v>
+        <v>126</v>
       </c>
       <c r="D55" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Ari Schifman   E2</v>
+        <v>Rajka Smiljanić   4.724</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B56" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>14</v>
+        <v>179</v>
       </c>
       <c r="D56" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Will Sheffield   W4</v>
+        <v>Madeline Smith   W5</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>129</v>
+        <v>103</v>
       </c>
       <c r="B57" t="s">
-        <v>130</v>
+        <v>104</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>131</v>
+        <v>105</v>
       </c>
       <c r="D57" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Rajka Smiljanić   4.724</v>
+        <v>Steve Wechsler   4.702</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>9</v>
+        <v>88</v>
       </c>
       <c r="B58" t="s">
-        <v>10</v>
+        <v>89</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>185</v>
+        <v>90</v>
       </c>
       <c r="D58" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Madeline Smith   W5</v>
+        <v>Debbie White   4.620</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>106</v>
+        <v>73</v>
       </c>
       <c r="B59" t="s">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
       <c r="D59" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Steve Wechsler   4.702</v>
+        <v>Elijah Wilder   E11</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>88</v>
+        <v>143</v>
       </c>
       <c r="B60" t="s">
-        <v>89</v>
+        <v>144</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="D60" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Debbie White   4.620</v>
+        <v>Tony Woodbury   4.738</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
       <c r="B61" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="D61" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Elijah Wilder   E11</v>
+        <v>Michael Wynne   4.626</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>148</v>
+        <v>17</v>
       </c>
       <c r="B62" t="s">
-        <v>149</v>
+        <v>18</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>150</v>
+        <v>19</v>
       </c>
       <c r="D62" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Tony Woodbury   4.738</v>
+        <v>Qing Yao   W6</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="B63" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="D63" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Michael Wynne   4.626</v>
+        <v>Hongli Zhan   (NA)</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B64" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D64" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Qing Yao   W6</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>78</v>
-      </c>
-      <c r="B65" t="s">
-        <v>79</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D65" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Hongli Zhan   (NA)</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>45</v>
-      </c>
-      <c r="B66" t="s">
-        <v>46</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D66" s="4" t="str">
-        <f t="shared" si="1"/>
         <v>Asher Zheng   W3</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D66">
-    <sortCondition ref="B3:B66"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D64">
+    <sortCondition ref="B3:B64"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates for Fall 2026
</commit_message>
<xml_diff>
--- a/people.xlsx
+++ b/people.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jessicaalexander/github/rlp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B09CE8DC-D989-A247-B4C4-409AAF426A9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3815E124-8396-654F-9483-EC5EFF4D2E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7620" yWindow="680" windowWidth="20820" windowHeight="15740" xr2:uid="{59A264FB-7A95-E842-AEEA-C35557593B53}"/>
+    <workbookView xWindow="12580" yWindow="680" windowWidth="15860" windowHeight="15740" xr2:uid="{59A264FB-7A95-E842-AEEA-C35557593B53}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="177">
   <si>
     <t>Baorian</t>
   </si>
@@ -64,12 +64,6 @@
     <t>W2</t>
   </si>
   <si>
-    <t>Madeline</t>
-  </si>
-  <si>
-    <t>Smith</t>
-  </si>
-  <si>
     <t>W3</t>
   </si>
   <si>
@@ -199,30 +193,12 @@
     <t>E3</t>
   </si>
   <si>
-    <t>Gabriella</t>
-  </si>
-  <si>
-    <t>Chronis</t>
-  </si>
-  <si>
-    <t>E4</t>
-  </si>
-  <si>
     <t>Masha</t>
   </si>
   <si>
     <t>Cheremisinova</t>
   </si>
   <si>
-    <t>E5</t>
-  </si>
-  <si>
-    <t>Sooji</t>
-  </si>
-  <si>
-    <t>E6</t>
-  </si>
-  <si>
     <t>Teagan</t>
   </si>
   <si>
@@ -271,18 +247,12 @@
     <t>Santamaria Soto</t>
   </si>
   <si>
-    <t>Hongli</t>
-  </si>
-  <si>
     <t>Zhan</t>
   </si>
   <si>
     <t>(NA)</t>
   </si>
   <si>
-    <t>E12</t>
-  </si>
-  <si>
     <t>Don</t>
   </si>
   <si>
@@ -547,12 +517,6 @@
     <t>Rojas</t>
   </si>
   <si>
-    <t>Yejin</t>
-  </si>
-  <si>
-    <t>Cho</t>
-  </si>
-  <si>
     <t>WCP 4.134</t>
   </si>
   <si>
@@ -565,15 +529,6 @@
     <t>4.434</t>
   </si>
   <si>
-    <t>4.110/W5</t>
-  </si>
-  <si>
-    <t>Sarah</t>
-  </si>
-  <si>
-    <t>Ransom Laud</t>
-  </si>
-  <si>
     <t>W5</t>
   </si>
   <si>
@@ -593,6 +548,24 @@
   </si>
   <si>
     <t>4.426</t>
+  </si>
+  <si>
+    <t>4.110/E4</t>
+  </si>
+  <si>
+    <t>Chan</t>
+  </si>
+  <si>
+    <t>Young Jung</t>
+  </si>
+  <si>
+    <t>Bowen</t>
+  </si>
+  <si>
+    <t>Yang</t>
+  </si>
+  <si>
+    <t>Haoran</t>
   </si>
 </sst>
 </file>
@@ -963,7 +936,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17483530-688E-B14A-9F3B-5498A1C19FFD}">
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="10.83203125" style="1"/>
@@ -972,30 +945,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="B2" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="D2" s="4" t="str">
-        <f t="shared" ref="D2:D36" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
+        <f t="shared" ref="D2:D33" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
         <v>Akshay Aitha   4.706</v>
       </c>
     </row>
@@ -1007,22 +980,22 @@
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>176</v>
+        <v>4</v>
       </c>
       <c r="D3" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Jess Alexander   4.110/W5</v>
+        <v>Jess Alexander   4.110</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="D4" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1031,13 +1004,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="B5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="D5" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1046,13 +1019,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D6" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1061,13 +1034,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B7" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="D7" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1076,13 +1049,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="B8" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="D8" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1106,13 +1079,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="B10" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D10" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1121,13 +1094,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="B11" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D11" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1136,817 +1109,772 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="D12" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Masha Cheremisinova   E5</v>
+        <v>Masha Cheremisinova   (NA)</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B13" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="D13" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Yejin Cho   (NA)</v>
+        <v>Caitlin Coons   E10</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>103</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>104</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="D14" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Gabriella Chronis   E4</v>
+        <v>Megan Crowhurst   4.712</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>180</v>
+        <v>141</v>
       </c>
       <c r="B15" t="s">
-        <v>181</v>
+        <v>140</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>72</v>
+        <v>160</v>
       </c>
       <c r="D15" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Caitlin Coons   E10</v>
+        <v>Meg Davidson   WCP 4.134</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>113</v>
+        <v>168</v>
       </c>
       <c r="B16" t="s">
-        <v>114</v>
+        <v>169</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>115</v>
+        <v>170</v>
       </c>
       <c r="D16" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Megan Crowhurst   4.712</v>
+        <v>Kristie Denlinger   4.426</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>151</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>150</v>
+        <v>14</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="D17" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Meg Davidson   WCP 4.134</v>
+        <v>Sampada Deshpande   4.434</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>183</v>
+        <v>130</v>
       </c>
       <c r="B18" t="s">
-        <v>184</v>
+        <v>131</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>185</v>
+        <v>132</v>
       </c>
       <c r="D18" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Kristie Denlinger   4.426</v>
+        <v>Pattie Epps   4.736</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="B19" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>175</v>
+        <v>56</v>
       </c>
       <c r="D19" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Sampada Deshpande   4.434</v>
+        <v>Teagan Esther   E7</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="B20" t="s">
-        <v>141</v>
+        <v>76</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>142</v>
+        <v>77</v>
       </c>
       <c r="D20" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Pattie Epps   4.736</v>
+        <v>James Fazio   4.622</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D21" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Teagan Esther   E7</v>
+        <v>Gabriel Gallinate   E8</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>87</v>
+        <v>30</v>
       </c>
       <c r="D22" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>James Fazio   4.622</v>
+        <v>Barrett Hamp   W12</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="D23" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Gabriel Gallinate   E8</v>
+        <v>Leticia Hanada   W10</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="D24" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Barrett Hamp   W12</v>
+        <v>Ethan Hartzell   E3</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>156</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>157</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="D25" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Leticia Hanada   W10</v>
+        <v>Juan Pablo Jáuregui Magrina   (NA)</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>154</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>155</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="D26" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Ethan Hartzell   E3</v>
+        <v>Anushri Kartik-Narajan   4.110/E4</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>166</v>
+        <v>90</v>
       </c>
       <c r="B27" t="s">
-        <v>167</v>
+        <v>91</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="D27" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Juan Pablo Jáuregui Magrina   (NA)</v>
+        <v>Danny Law   4.432</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>164</v>
+        <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>165</v>
+        <v>85</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="D28" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Anushri Kartik-Narajan   4.110</v>
+        <v>Rebecca Le Borgne   4.624</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="B29" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="D29" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Danny Law   4.432</v>
+        <v>Jessy Li   4.728</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>123</v>
       </c>
       <c r="B30" t="s">
-        <v>95</v>
+        <v>124</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="D30" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Rebecca Le Borgne   4.624</v>
+        <v>Fernando Llanos   4.730</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="B31" t="s">
-        <v>23</v>
+        <v>88</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="D31" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Sooji Lee   E6</v>
+        <v>Kyle Mahowald   4.430</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>130</v>
+        <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>131</v>
+        <v>38</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>132</v>
+        <v>39</v>
       </c>
       <c r="D32" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Jessy Li   4.728</v>
+        <v>Rebecca Marcus   4.304C</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B33" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D33" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Fernando Llanos   4.730</v>
+        <v>Richard Meier   4.732</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="B34" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="D34" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Kyle Mahowald   4.430</v>
+        <f t="shared" ref="D34:D62" si="1">CONCATENATE(A34, " ", B34, "   ", C34)</f>
+        <v>Don Miller   4.618</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="B35" t="s">
-        <v>40</v>
+        <v>146</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
       <c r="D35" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Rebecca Marcus   4.304C</v>
+        <f t="shared" si="1"/>
+        <v>Kanishka Misra   4.428</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>136</v>
+        <v>167</v>
       </c>
       <c r="B36" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>138</v>
+        <v>5</v>
       </c>
       <c r="D36" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Richard Meier   4.732</v>
+        <f t="shared" si="1"/>
+        <v>Kaijie Mo   W1</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>82</v>
+        <v>117</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>118</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="D37" s="4" t="str">
-        <f t="shared" ref="D37:D65" si="1">CONCATENATE(A37, " ", B37, "   ", C37)</f>
-        <v>Don Miller   4.618</v>
+        <f t="shared" si="1"/>
+        <v>Scott Myers   4.726</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>155</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>156</v>
+        <v>35</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="D38" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Kanishka Misra   4.428</v>
+        <v>Lillian Nguyen   FD</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>182</v>
+        <v>0</v>
       </c>
       <c r="B39" t="s">
-        <v>159</v>
+        <v>1</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>5</v>
+        <v>162</v>
       </c>
       <c r="D39" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Kaijie Mo   W1</v>
+        <v>Baorian Nuchged   4.110/W11</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="B40" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>129</v>
       </c>
       <c r="D40" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Scott Myers   4.726</v>
+        <v>Karol Obert   4.734</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>36</v>
+        <v>96</v>
       </c>
       <c r="B41" t="s">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="D41" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lillian Nguyen   FD</v>
+        <v>Corrine Occhino   4.704</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="B42" t="s">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>174</v>
+        <v>23</v>
       </c>
       <c r="D42" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Baorian Nuchged   4.110/W11</v>
+        <v>Lee Orfila   W8</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>152</v>
+        <v>18</v>
       </c>
       <c r="B43" t="s">
-        <v>153</v>
+        <v>19</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>139</v>
+        <v>20</v>
       </c>
       <c r="D43" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Karol Obert   4.734</v>
+        <v>Youn-Gyu Park   W7</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>106</v>
+        <v>63</v>
       </c>
       <c r="B44" t="s">
-        <v>107</v>
+        <v>19</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>108</v>
+        <v>71</v>
       </c>
       <c r="D44" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Corrine Occhino   4.704</v>
+        <v>SeYeon Park   (NA)</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>23</v>
+        <v>100</v>
       </c>
       <c r="B45" t="s">
-        <v>24</v>
+        <v>106</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>25</v>
+        <v>107</v>
       </c>
       <c r="D45" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lee Orfila   W8</v>
+        <v>David Quinto-Pozos   4.714</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B46" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D46" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Youn-Gyu Park   W7</v>
+        <v>Ben Rapstine   4.304D</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>71</v>
+        <v>158</v>
       </c>
       <c r="B47" t="s">
-        <v>21</v>
+        <v>159</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="D47" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>SeYeon Park   (NA)</v>
+        <v>Oscar Rojas   E8</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="B48" t="s">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>117</v>
+        <v>71</v>
       </c>
       <c r="D48" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>David Quinto-Pozos   4.714</v>
+        <v>Catalina Santamaria Soto   (NA)</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>177</v>
+        <v>31</v>
       </c>
       <c r="B49" t="s">
-        <v>178</v>
+        <v>32</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="D49" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Sarah Ransom Laud   (NA)</v>
+        <v>Jefferson Saransig   W13</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>42</v>
+        <v>150</v>
       </c>
       <c r="B50" t="s">
-        <v>43</v>
+        <v>151</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D50" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Ben Rapstine   4.304D</v>
+        <v>Ari Schifman   E2</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>168</v>
+        <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>169</v>
+        <v>11</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D51" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Oscar Rojas   E8</v>
+        <v>Will Sheffield   (NA)</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>76</v>
+        <v>114</v>
       </c>
       <c r="B52" t="s">
-        <v>77</v>
+        <v>115</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="D52" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Catalina Santamaria Soto   E12</v>
+        <v>Rajka Smiljanić   4.724</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>33</v>
+        <v>93</v>
       </c>
       <c r="B53" t="s">
-        <v>34</v>
+        <v>94</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="D53" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Jefferson Saransig   W13</v>
+        <v>Steve Wechsler   4.702</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>160</v>
+        <v>78</v>
       </c>
       <c r="B54" t="s">
-        <v>161</v>
+        <v>79</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="D54" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Ari Schifman   E2</v>
+        <v>Debbie White   4.620</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>13</v>
+        <v>66</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="D55" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Will Sheffield   W4</v>
+        <v>Elijah Wilder   E11</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="B56" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="D56" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Rajka Smiljanić   4.724</v>
+        <v>Tony Woodbury   4.738</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>9</v>
+        <v>81</v>
       </c>
       <c r="B57" t="s">
-        <v>10</v>
+        <v>82</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>179</v>
+        <v>83</v>
       </c>
       <c r="D57" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Madeline Smith   W5</v>
+        <v>Michael Wynne   4.626</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>103</v>
+        <v>174</v>
       </c>
       <c r="B58" t="s">
-        <v>104</v>
+        <v>175</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>105</v>
+        <v>163</v>
       </c>
       <c r="D58" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Steve Wechsler   4.702</v>
+        <v>Bowen Yang   4.434</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>88</v>
+        <v>15</v>
       </c>
       <c r="B59" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>90</v>
+        <v>17</v>
       </c>
       <c r="D59" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Debbie White   4.620</v>
+        <v>Qing Yao   W6</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>73</v>
+        <v>172</v>
       </c>
       <c r="B60" t="s">
-        <v>74</v>
+        <v>173</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>75</v>
+        <v>12</v>
       </c>
       <c r="D60" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Elijah Wilder   E11</v>
+        <v>Chan Young Jung   W4</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>143</v>
+        <v>176</v>
       </c>
       <c r="B61" t="s">
-        <v>144</v>
+        <v>70</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="D61" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Tony Woodbury   4.738</v>
+        <v>Haoran Zhan   W5</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>91</v>
+        <v>43</v>
       </c>
       <c r="B62" t="s">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="D62" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Michael Wynne   4.626</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>17</v>
-      </c>
-      <c r="B63" t="s">
-        <v>18</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D63" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Qing Yao   W6</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>78</v>
-      </c>
-      <c r="B64" t="s">
-        <v>79</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D64" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Hongli Zhan   (NA)</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>45</v>
-      </c>
-      <c r="B65" t="s">
-        <v>46</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D65" s="4" t="str">
-        <f t="shared" si="1"/>
         <v>Asher Zheng   W3</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D65">
-    <sortCondition ref="B3:B65"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D62">
+    <sortCondition ref="B3:B62"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Additional updates for Fall 2026
</commit_message>
<xml_diff>
--- a/people.xlsx
+++ b/people.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jessicaalexander/github/rlp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3815E124-8396-654F-9483-EC5EFF4D2E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE108E9-0553-C442-9A8A-09B5E42D9FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12580" yWindow="680" windowWidth="15860" windowHeight="15740" xr2:uid="{59A264FB-7A95-E842-AEEA-C35557593B53}"/>
+    <workbookView xWindow="2900" yWindow="680" windowWidth="15860" windowHeight="15680" xr2:uid="{59A264FB-7A95-E842-AEEA-C35557593B53}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="180">
   <si>
     <t>Baorian</t>
   </si>
@@ -118,9 +118,6 @@
     <t>Hanada</t>
   </si>
   <si>
-    <t>W10</t>
-  </si>
-  <si>
     <t>Barrett</t>
   </si>
   <si>
@@ -136,9 +133,6 @@
     <t>Saransig</t>
   </si>
   <si>
-    <t>W13</t>
-  </si>
-  <si>
     <t>Lillian</t>
   </si>
   <si>
@@ -550,9 +544,6 @@
     <t>4.426</t>
   </si>
   <si>
-    <t>4.110/E4</t>
-  </si>
-  <si>
     <t>Chan</t>
   </si>
   <si>
@@ -562,10 +553,28 @@
     <t>Bowen</t>
   </si>
   <si>
-    <t>Yang</t>
-  </si>
-  <si>
     <t>Haoran</t>
+  </si>
+  <si>
+    <t>Jiang</t>
+  </si>
+  <si>
+    <t>Kamath</t>
+  </si>
+  <si>
+    <t>Gaurav</t>
+  </si>
+  <si>
+    <t>4.110/E12</t>
+  </si>
+  <si>
+    <t>E4</t>
+  </si>
+  <si>
+    <t>E5</t>
+  </si>
+  <si>
+    <t>E6</t>
   </si>
 </sst>
 </file>
@@ -626,7 +635,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -936,7 +966,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17483530-688E-B14A-9F3B-5498A1C19FFD}">
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="10.83203125" style="1"/>
@@ -945,30 +975,30 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D2" s="4" t="str">
-        <f t="shared" ref="D2:D33" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
+        <f t="shared" ref="D2:D35" si="0">CONCATENATE(A2, " ", B2, "   ", C2)</f>
         <v>Akshay Aitha   4.706</v>
       </c>
     </row>
@@ -989,13 +1019,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>110</v>
       </c>
       <c r="D4" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1004,13 +1034,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="D5" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1019,13 +1049,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="D6" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1034,13 +1064,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="D7" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1049,13 +1079,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="B8" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="D8" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1079,13 +1109,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D10" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1094,28 +1124,28 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B11" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>24</v>
+        <v>179</v>
       </c>
       <c r="D11" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Thiago Cardoso Aguiar   W9</v>
+        <v>Thiago Cardoso Aguiar   E6</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D12" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1124,13 +1154,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B13" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D13" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1139,13 +1169,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" t="s">
+        <v>102</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="B14" t="s">
-        <v>104</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="D14" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1154,13 +1184,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B15" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D15" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1169,13 +1199,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>166</v>
+      </c>
+      <c r="B16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="B16" t="s">
-        <v>169</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>170</v>
       </c>
       <c r="D16" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1190,7 +1220,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D17" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1199,13 +1229,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>128</v>
+      </c>
+      <c r="B18" t="s">
+        <v>129</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="B18" t="s">
-        <v>131</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="D18" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1214,13 +1244,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="B19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="D19" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1229,13 +1259,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="B20" t="s">
-        <v>76</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="D20" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1244,13 +1274,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B21" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="B21" t="s">
-        <v>58</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="D21" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1259,13 +1289,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
         <v>28</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="D22" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1280,22 +1310,22 @@
         <v>26</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>27</v>
+        <v>178</v>
       </c>
       <c r="D23" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Leticia Hanada   W10</v>
+        <v>Leticia Hanada   E5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="B24" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="D24" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1304,13 +1334,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B25" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D25" s="4" t="str">
         <f t="shared" si="0"/>
@@ -1319,562 +1349,577 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="B26" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="D26" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Anushri Kartik-Narajan   4.110/E4</v>
+        <f>CONCATENATE(A26, " ", B26, "   ", C26)</f>
+        <v>Bowen Jiang   4.434</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>90</v>
+        <v>175</v>
       </c>
       <c r="B27" t="s">
-        <v>91</v>
+        <v>174</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="D27" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Danny Law   4.432</v>
+        <f>CONCATENATE(A27, " ", B27, "   ", C27)</f>
+        <v>Gaurav Kamath   W9</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>152</v>
       </c>
       <c r="B28" t="s">
-        <v>85</v>
+        <v>153</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>84</v>
+        <v>176</v>
       </c>
       <c r="D28" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Rebecca Le Borgne   4.624</v>
+        <v>Anushri Kartik-Narajan   4.110/E12</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="B29" t="s">
-        <v>121</v>
+        <v>89</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>122</v>
+        <v>90</v>
       </c>
       <c r="D29" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Jessy Li   4.728</v>
+        <v>Danny Law   4.432</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>123</v>
+        <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>124</v>
+        <v>83</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>125</v>
+        <v>82</v>
       </c>
       <c r="D30" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Fernando Llanos   4.730</v>
+        <v>Rebecca Le Borgne   4.624</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="B31" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="D31" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Kyle Mahowald   4.430</v>
+        <v>Jessy Li   4.728</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>121</v>
       </c>
       <c r="B32" t="s">
-        <v>38</v>
+        <v>122</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>39</v>
+        <v>123</v>
       </c>
       <c r="D32" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Rebecca Marcus   4.304C</v>
+        <v>Fernando Llanos   4.730</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>126</v>
+        <v>85</v>
       </c>
       <c r="B33" t="s">
-        <v>127</v>
+        <v>86</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>128</v>
+        <v>87</v>
       </c>
       <c r="D33" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>Richard Meier   4.732</v>
+        <v>Kyle Mahowald   4.430</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="D34" s="4" t="str">
-        <f t="shared" ref="D34:D62" si="1">CONCATENATE(A34, " ", B34, "   ", C34)</f>
-        <v>Don Miller   4.618</v>
+        <f t="shared" si="0"/>
+        <v>Rebecca Marcus   4.304C</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>145</v>
+        <v>124</v>
       </c>
       <c r="B35" t="s">
-        <v>146</v>
+        <v>125</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>86</v>
+        <v>126</v>
       </c>
       <c r="D35" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Kanishka Misra   4.428</v>
+        <f t="shared" si="0"/>
+        <v>Richard Meier   4.732</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>167</v>
+        <v>70</v>
       </c>
       <c r="B36" t="s">
-        <v>149</v>
+        <v>71</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>5</v>
+        <v>72</v>
       </c>
       <c r="D36" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Kaijie Mo   W1</v>
+        <f t="shared" ref="D36:D63" si="1">CONCATENATE(A36, " ", B36, "   ", C36)</f>
+        <v>Don Miller   4.618</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>117</v>
+        <v>143</v>
       </c>
       <c r="B37" t="s">
-        <v>118</v>
+        <v>144</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="D37" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Scott Myers   4.726</v>
+        <v>Kanishka Misra   4.428</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>34</v>
+        <v>165</v>
       </c>
       <c r="B38" t="s">
-        <v>35</v>
+        <v>147</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="D38" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lillian Nguyen   FD</v>
+        <v>Kaijie Mo   W1</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="B39" t="s">
-        <v>1</v>
+        <v>116</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>162</v>
+        <v>117</v>
       </c>
       <c r="D39" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Baorian Nuchged   4.110/W11</v>
+        <v>Scott Myers   4.726</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>142</v>
+        <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>143</v>
+        <v>33</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>129</v>
+        <v>34</v>
       </c>
       <c r="D40" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Karol Obert   4.734</v>
+        <v>Lillian Nguyen   FD</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>97</v>
+        <v>1</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>98</v>
+        <v>160</v>
       </c>
       <c r="D41" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Corrine Occhino   4.704</v>
+        <v>Baorian Nuchged   4.110/W11</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>21</v>
+        <v>140</v>
       </c>
       <c r="B42" t="s">
-        <v>22</v>
+        <v>141</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>23</v>
+        <v>127</v>
       </c>
       <c r="D42" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Lee Orfila   W8</v>
+        <v>Karol Obert   4.734</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="B43" t="s">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="D43" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Youn-Gyu Park   W7</v>
+        <v>Corrine Occhino   4.704</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="B44" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="D44" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>SeYeon Park   (NA)</v>
+        <v>Lee Orfila   W8</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="B45" t="s">
-        <v>106</v>
+        <v>19</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>107</v>
+        <v>20</v>
       </c>
       <c r="D45" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>David Quinto-Pozos   4.714</v>
+        <v>Youn-Gyu Park   W7</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="B46" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="D46" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Ben Rapstine   4.304D</v>
+        <v>SeYeon Park   (NA)</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>158</v>
+        <v>98</v>
       </c>
       <c r="B47" t="s">
-        <v>159</v>
+        <v>104</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>59</v>
+        <v>105</v>
       </c>
       <c r="D47" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Oscar Rojas   E8</v>
+        <v>David Quinto-Pozos   4.714</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="B48" t="s">
-        <v>69</v>
+        <v>39</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="D48" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Catalina Santamaria Soto   (NA)</v>
+        <v>Ben Rapstine   4.304D</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>31</v>
+        <v>156</v>
       </c>
       <c r="B49" t="s">
-        <v>32</v>
+        <v>157</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="D49" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Jefferson Saransig   W13</v>
+        <v>Oscar Rojas   E8</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>150</v>
+        <v>66</v>
       </c>
       <c r="B50" t="s">
-        <v>151</v>
+        <v>67</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="D50" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Ari Schifman   E2</v>
+        <v>Catalina Santamaria Soto   (NA)</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B51" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>71</v>
+        <v>177</v>
       </c>
       <c r="D51" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Will Sheffield   (NA)</v>
+        <v>Jefferson Saransig   E4</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="B52" t="s">
-        <v>115</v>
+        <v>149</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>116</v>
+        <v>46</v>
       </c>
       <c r="D52" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Rajka Smiljanić   4.724</v>
+        <v>Ari Schifman   E2</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>93</v>
+        <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>94</v>
+        <v>11</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="D53" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Steve Wechsler   4.702</v>
+        <v>Will Sheffield   (NA)</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="B54" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="D54" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Debbie White   4.620</v>
+        <v>Rajka Smiljanić   4.724</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
       <c r="B55" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="D55" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Elijah Wilder   E11</v>
+        <v>Steve Wechsler   4.702</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>133</v>
+        <v>76</v>
       </c>
       <c r="B56" t="s">
-        <v>134</v>
+        <v>77</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>135</v>
+        <v>78</v>
       </c>
       <c r="D56" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Tony Woodbury   4.738</v>
+        <v>Debbie White   4.620</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="B57" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="D57" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Michael Wynne   4.626</v>
+        <v>Elijah Wilder   E11</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>174</v>
+        <v>131</v>
       </c>
       <c r="B58" t="s">
-        <v>175</v>
+        <v>132</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
       <c r="D58" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Bowen Yang   4.434</v>
+        <v>Tony Woodbury   4.738</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>15</v>
+        <v>79</v>
       </c>
       <c r="B59" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>17</v>
+        <v>81</v>
       </c>
       <c r="D59" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Qing Yao   W6</v>
+        <v>Michael Wynne   4.626</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>172</v>
+        <v>15</v>
       </c>
       <c r="B60" t="s">
-        <v>173</v>
+        <v>16</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D60" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Chan Young Jung   W4</v>
+        <v>Qing Yao   W6</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="B61" t="s">
-        <v>70</v>
+        <v>170</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>164</v>
+        <v>12</v>
       </c>
       <c r="D61" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Haoran Zhan   W5</v>
+        <v>Chan Young Jung   W4</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>43</v>
+        <v>172</v>
       </c>
       <c r="B62" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="C62" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D62" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>Haoran Zhan   W5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>41</v>
+      </c>
+      <c r="B63" t="s">
+        <v>42</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D62" s="4" t="str">
+      <c r="D63" s="4" t="str">
         <f t="shared" si="1"/>
         <v>Asher Zheng   W3</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D62">
-    <sortCondition ref="B3:B62"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D63">
+    <sortCondition ref="B3:B63"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>